<commit_message>
Atualização automática: Dispersão KM por Motorista.xlsx
</commit_message>
<xml_diff>
--- a/Dispersão KM por Motorista.xlsx
+++ b/Dispersão KM por Motorista.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="Ra1e95ffa0835403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Export" sheetId="1" r:id="Rdb02bc131ebe4f4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -130,6 +130,19 @@
     </x:row>
     <x:row>
       <x:c s="8">
+        <x:v>317</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>CARLOS  SANTO</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.20817843866171004</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
         <x:v>331</x:v>
       </x:c>
       <x:c t="inlineStr">
@@ -177,7 +190,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.088908845981140683</x:v>
+        <x:v>0.15909490512192814</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -203,7 +216,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.084288052373158839</x:v>
+        <x:v>0.17338273892234057</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -216,7 +229,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.14049909020015594</x:v>
+        <x:v>0.14948761047551917</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -242,7 +255,20 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.20505772402418909</x:v>
+        <x:v>0.17535958157780018</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>ISMAEL  SIQUEIRA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.18034586878945924</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -268,7 +294,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.079526353143326789</x:v>
+        <x:v>0.19428181458999338</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -294,7 +320,33 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.032369974540469526</x:v>
+        <x:v>0.077048396064183233</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>323</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JOSE  RIQUELME</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.22168601365158036</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>233</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>JUNIOR  SILVA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.34730538922155696</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -333,7 +385,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.15341856586992786</x:v>
+        <x:v>0.1897572170552</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -385,7 +437,7 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.35823429541595919</x:v>
+        <x:v>0.24698310539018498</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -398,7 +450,33 @@
         </x:is>
       </x:c>
       <x:c s="9">
-        <x:v>0.40120329322355919</x:v>
+        <x:v>0.24028505450301707</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>268</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>NIY  OLIVEIRA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.32108513318381515</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>REGIANDRO  MOREIRA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.87106297166379076</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -412,6 +490,19 @@
       </x:c>
       <x:c s="9">
         <x:v>0.58279220779220786</x:v>
+      </x:c>
+    </x:row>
+    <x:row>
+      <x:c s="8">
+        <x:v>288</x:v>
+      </x:c>
+      <x:c t="inlineStr">
+        <x:is>
+          <x:t>ROWILSON  PEREIRA</x:t>
+        </x:is>
+      </x:c>
+      <x:c s="9">
+        <x:v>0.40503875968992253</x:v>
       </x:c>
     </x:row>
     <x:row>
@@ -448,7 +539,7 @@
       </x:c>
       <x:c s="1"/>
       <x:c s="10">
-        <x:v>0.16667691459377543</x:v>
+        <x:v>0.24000826901874306</x:v>
       </x:c>
     </x:row>
     <x:row/>
@@ -460,7 +551,7 @@
 Revenda é GranDourados
 Frota é Padronizada
 Ano é 2026
-Date é igual a ou está depois de 01/09/2026 e está antes de 04/09/2026
+Date é igual a ou está depois de 01/09/2026 e está antes de 06/09/2026
 Taxa de Dispersão é Até 100%
 Check Dispersão KM é Sim
 Tipo Dispersão KM é Positiva

</xml_diff>